<commit_message>
Enhance ML capabilities by adding lightgbm and catboost dependencies in pyproject.toml and uv.lock. Implement ML pipeline scheduler in main.py for daily execution. Update audio conversion to use ffmpeg, removing pydub dependency. Revise EDA notebook for churn analysis and streamline model files by removing outdated models and scripts.
</commit_message>
<xml_diff>
--- a/data/test_dataset_15_accounts.xlsx
+++ b/data/test_dataset_15_accounts.xlsx
@@ -7,14 +7,14 @@
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Accounts" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="282" uniqueCount="162">
   <si>
     <t>name</t>
   </si>
@@ -52,6 +52,12 @@
     <t>renewal_stage</t>
   </si>
   <si>
+    <t>sentiment_score</t>
+  </si>
+  <si>
+    <t>sentiment_category</t>
+  </si>
+  <si>
     <t>licenses_used</t>
   </si>
   <si>
@@ -91,12 +97,6 @@
     <t>churn_probability</t>
   </si>
   <si>
-    <t>sentiment_score</t>
-  </si>
-  <si>
-    <t>sentiment_category</t>
-  </si>
-  <si>
     <t>TechCorp Solutions</t>
   </si>
   <si>
@@ -241,94 +241,85 @@
     <t>Large</t>
   </si>
   <si>
-    <t>2024-07-21</t>
-  </si>
-  <si>
-    <t>2024-05-30</t>
-  </si>
-  <si>
-    <t>2024-09-30</t>
-  </si>
-  <si>
-    <t>2025-06-26</t>
-  </si>
-  <si>
-    <t>2025-05-13</t>
-  </si>
-  <si>
-    <t>2024-07-01</t>
-  </si>
-  <si>
-    <t>2024-05-16</t>
-  </si>
-  <si>
-    <t>2025-03-05</t>
-  </si>
-  <si>
-    <t>2024-09-07</t>
-  </si>
-  <si>
-    <t>2025-05-25</t>
-  </si>
-  <si>
-    <t>2024-04-01</t>
-  </si>
-  <si>
-    <t>2024-12-01</t>
-  </si>
-  <si>
-    <t>2024-04-20</t>
-  </si>
-  <si>
-    <t>2024-04-17</t>
-  </si>
-  <si>
-    <t>2025-02-23</t>
-  </si>
-  <si>
-    <t>2025-07-21</t>
-  </si>
-  <si>
-    <t>2025-05-30</t>
-  </si>
-  <si>
-    <t>2025-09-30</t>
-  </si>
-  <si>
-    <t>2026-06-26</t>
-  </si>
-  <si>
-    <t>2026-05-13</t>
-  </si>
-  <si>
-    <t>2025-07-01</t>
-  </si>
-  <si>
-    <t>2025-05-16</t>
-  </si>
-  <si>
-    <t>2026-03-05</t>
-  </si>
-  <si>
-    <t>2025-09-07</t>
-  </si>
-  <si>
-    <t>2026-05-25</t>
-  </si>
-  <si>
-    <t>2025-04-01</t>
-  </si>
-  <si>
-    <t>2025-12-01</t>
-  </si>
-  <si>
-    <t>2025-04-20</t>
-  </si>
-  <si>
-    <t>2025-04-17</t>
-  </si>
-  <si>
-    <t>2026-02-23</t>
+    <t>2025-02-21</t>
+  </si>
+  <si>
+    <t>2025-12-23</t>
+  </si>
+  <si>
+    <t>2026-01-02</t>
+  </si>
+  <si>
+    <t>2026-01-07</t>
+  </si>
+  <si>
+    <t>2025-08-25</t>
+  </si>
+  <si>
+    <t>2025-09-04</t>
+  </si>
+  <si>
+    <t>2025-09-14</t>
+  </si>
+  <si>
+    <t>2025-04-27</t>
+  </si>
+  <si>
+    <t>2025-05-07</t>
+  </si>
+  <si>
+    <t>2025-05-17</t>
+  </si>
+  <si>
+    <t>2025-05-27</t>
+  </si>
+  <si>
+    <t>2025-06-06</t>
+  </si>
+  <si>
+    <t>2025-06-16</t>
+  </si>
+  <si>
+    <t>2025-11-23</t>
+  </si>
+  <si>
+    <t>2026-01-22</t>
+  </si>
+  <si>
+    <t>2026-12-23</t>
+  </si>
+  <si>
+    <t>2027-01-02</t>
+  </si>
+  <si>
+    <t>2027-01-07</t>
+  </si>
+  <si>
+    <t>2026-08-25</t>
+  </si>
+  <si>
+    <t>2026-09-04</t>
+  </si>
+  <si>
+    <t>2026-09-14</t>
+  </si>
+  <si>
+    <t>2026-04-27</t>
+  </si>
+  <si>
+    <t>2026-05-07</t>
+  </si>
+  <si>
+    <t>2026-05-17</t>
+  </si>
+  <si>
+    <t>2026-05-27</t>
+  </si>
+  <si>
+    <t>2026-06-06</t>
+  </si>
+  <si>
+    <t>2026-06-16</t>
   </si>
   <si>
     <t>2026-01-28 15:24:16</t>
@@ -367,12 +358,12 @@
     <t>2026-02-14 15:24:16</t>
   </si>
   <si>
+    <t>renewed</t>
+  </si>
+  <si>
     <t>active</t>
   </si>
   <si>
-    <t>renewed</t>
-  </si>
-  <si>
     <t>t60</t>
   </si>
   <si>
@@ -380,6 +371,21 @@
   </si>
   <si>
     <t>t90</t>
+  </si>
+  <si>
+    <t>very_positive</t>
+  </si>
+  <si>
+    <t>positive</t>
+  </si>
+  <si>
+    <t>neutral</t>
+  </si>
+  <si>
+    <t>negative</t>
+  </si>
+  <si>
+    <t>very_negative</t>
   </si>
   <si>
     <t>Maria Lopez</t>
@@ -960,46 +966,64 @@
         <v>75</v>
       </c>
       <c r="H2" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="I2" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="J2" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="K2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="L2" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="M2">
+        <v>0.875</v>
+      </c>
+      <c r="N2" t="s">
+        <v>119</v>
+      </c>
+      <c r="O2">
         <v>124</v>
       </c>
-      <c r="N2">
+      <c r="P2">
         <v>140</v>
       </c>
-      <c r="O2">
+      <c r="Q2">
         <v>89</v>
       </c>
-      <c r="P2" t="s">
-        <v>122</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>129</v>
-      </c>
       <c r="R2" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="S2" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="T2" t="s">
-        <v>144</v>
+        <v>132</v>
       </c>
       <c r="U2" t="s">
-        <v>145</v>
+        <v>131</v>
+      </c>
+      <c r="V2" t="s">
+        <v>146</v>
+      </c>
+      <c r="W2" t="s">
+        <v>147</v>
+      </c>
+      <c r="X2">
+        <v>65</v>
+      </c>
+      <c r="Y2">
+        <v>35</v>
+      </c>
+      <c r="Z2">
+        <v>70</v>
+      </c>
+      <c r="AA2">
+        <v>0.25</v>
       </c>
     </row>
     <row r="3" spans="1:27">
@@ -1022,49 +1046,67 @@
         <v>16600.38</v>
       </c>
       <c r="G3" t="s">
+        <v>75</v>
+      </c>
+      <c r="H3" t="s">
         <v>76</v>
       </c>
-      <c r="H3" t="s">
-        <v>91</v>
-      </c>
       <c r="I3" t="s">
-        <v>91</v>
+        <v>76</v>
       </c>
       <c r="J3" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="K3" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="L3" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="M3">
+        <v>0.55</v>
+      </c>
+      <c r="N3" t="s">
+        <v>120</v>
+      </c>
+      <c r="O3">
         <v>143</v>
       </c>
-      <c r="N3">
+      <c r="P3">
         <v>169</v>
       </c>
-      <c r="O3">
+      <c r="Q3">
         <v>85</v>
       </c>
-      <c r="P3" t="s">
-        <v>123</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>129</v>
-      </c>
       <c r="R3" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="S3" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="T3" t="s">
-        <v>144</v>
+        <v>133</v>
       </c>
       <c r="U3" t="s">
+        <v>131</v>
+      </c>
+      <c r="V3" t="s">
         <v>146</v>
+      </c>
+      <c r="W3" t="s">
+        <v>148</v>
+      </c>
+      <c r="X3">
+        <v>65</v>
+      </c>
+      <c r="Y3">
+        <v>35</v>
+      </c>
+      <c r="Z3">
+        <v>70</v>
+      </c>
+      <c r="AA3">
+        <v>0.25</v>
       </c>
     </row>
     <row r="4" spans="1:27">
@@ -1087,49 +1129,67 @@
         <v>16100.95</v>
       </c>
       <c r="G4" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H4" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="I4" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="J4" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="K4" t="s">
+        <v>114</v>
+      </c>
+      <c r="L4" t="s">
         <v>117</v>
       </c>
-      <c r="L4" t="s">
-        <v>120</v>
-      </c>
       <c r="M4">
+        <v>0.05</v>
+      </c>
+      <c r="N4" t="s">
+        <v>121</v>
+      </c>
+      <c r="O4">
         <v>140</v>
       </c>
-      <c r="N4">
+      <c r="P4">
         <v>163</v>
       </c>
-      <c r="O4">
+      <c r="Q4">
         <v>86</v>
       </c>
-      <c r="P4" t="s">
-        <v>124</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>129</v>
-      </c>
       <c r="R4" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="S4" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="T4" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="U4" t="s">
-        <v>147</v>
+        <v>131</v>
+      </c>
+      <c r="V4" t="s">
+        <v>146</v>
+      </c>
+      <c r="W4" t="s">
+        <v>149</v>
+      </c>
+      <c r="X4">
+        <v>65</v>
+      </c>
+      <c r="Y4">
+        <v>35</v>
+      </c>
+      <c r="Z4">
+        <v>70</v>
+      </c>
+      <c r="AA4">
+        <v>0.25</v>
       </c>
     </row>
     <row r="5" spans="1:27">
@@ -1152,49 +1212,67 @@
         <v>29607.6</v>
       </c>
       <c r="G5" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="H5" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="I5" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="J5" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="K5" t="s">
+        <v>115</v>
+      </c>
+      <c r="L5" t="s">
         <v>117</v>
       </c>
-      <c r="L5" t="s">
-        <v>120</v>
-      </c>
       <c r="M5">
+        <v>-0.5</v>
+      </c>
+      <c r="N5" t="s">
+        <v>122</v>
+      </c>
+      <c r="O5">
         <v>36</v>
       </c>
-      <c r="N5">
+      <c r="P5">
         <v>51</v>
       </c>
-      <c r="O5">
+      <c r="Q5">
         <v>72</v>
       </c>
-      <c r="P5" t="s">
-        <v>124</v>
-      </c>
-      <c r="Q5" t="s">
-        <v>129</v>
-      </c>
       <c r="R5" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="S5" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="T5" t="s">
-        <v>144</v>
+        <v>135</v>
       </c>
       <c r="U5" t="s">
-        <v>148</v>
+        <v>131</v>
+      </c>
+      <c r="V5" t="s">
+        <v>146</v>
+      </c>
+      <c r="W5" t="s">
+        <v>150</v>
+      </c>
+      <c r="X5">
+        <v>65</v>
+      </c>
+      <c r="Y5">
+        <v>35</v>
+      </c>
+      <c r="Z5">
+        <v>70</v>
+      </c>
+      <c r="AA5">
+        <v>0.25</v>
       </c>
     </row>
     <row r="6" spans="1:27">
@@ -1217,49 +1295,67 @@
         <v>41528.6</v>
       </c>
       <c r="G6" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="H6" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="I6" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="J6" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="K6" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="L6" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="M6">
+        <v>-0.875</v>
+      </c>
+      <c r="N6" t="s">
+        <v>123</v>
+      </c>
+      <c r="O6">
         <v>70</v>
       </c>
-      <c r="N6">
+      <c r="P6">
         <v>113</v>
       </c>
-      <c r="O6">
+      <c r="Q6">
         <v>62</v>
       </c>
-      <c r="P6" t="s">
-        <v>123</v>
-      </c>
-      <c r="Q6" t="s">
-        <v>129</v>
-      </c>
       <c r="R6" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="S6" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="T6" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
       <c r="U6" t="s">
-        <v>149</v>
+        <v>131</v>
+      </c>
+      <c r="V6" t="s">
+        <v>146</v>
+      </c>
+      <c r="W6" t="s">
+        <v>151</v>
+      </c>
+      <c r="X6">
+        <v>65</v>
+      </c>
+      <c r="Y6">
+        <v>35</v>
+      </c>
+      <c r="Z6">
+        <v>70</v>
+      </c>
+      <c r="AA6">
+        <v>0.25</v>
       </c>
     </row>
     <row r="7" spans="1:27">
@@ -1282,49 +1378,67 @@
         <v>1622.41</v>
       </c>
       <c r="G7" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="H7" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="I7" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="J7" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="K7" t="s">
+        <v>115</v>
+      </c>
+      <c r="L7" t="s">
         <v>117</v>
       </c>
-      <c r="L7" t="s">
+      <c r="M7">
+        <v>0.55</v>
+      </c>
+      <c r="N7" t="s">
         <v>120</v>
       </c>
-      <c r="M7">
+      <c r="O7">
         <v>47</v>
       </c>
-      <c r="N7">
+      <c r="P7">
         <v>109</v>
       </c>
-      <c r="O7">
+      <c r="Q7">
         <v>44</v>
       </c>
-      <c r="P7" t="s">
-        <v>122</v>
-      </c>
-      <c r="Q7" t="s">
-        <v>129</v>
-      </c>
       <c r="R7" t="s">
-        <v>135</v>
+        <v>124</v>
       </c>
       <c r="S7" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="T7" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="U7" t="s">
-        <v>150</v>
+        <v>131</v>
+      </c>
+      <c r="V7" t="s">
+        <v>146</v>
+      </c>
+      <c r="W7" t="s">
+        <v>152</v>
+      </c>
+      <c r="X7">
+        <v>65</v>
+      </c>
+      <c r="Y7">
+        <v>35</v>
+      </c>
+      <c r="Z7">
+        <v>70</v>
+      </c>
+      <c r="AA7">
+        <v>0.25</v>
       </c>
     </row>
     <row r="8" spans="1:27">
@@ -1347,49 +1461,67 @@
         <v>20954.26</v>
       </c>
       <c r="G8" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="H8" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="I8" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="J8" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="K8" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="L8" t="s">
+        <v>118</v>
+      </c>
+      <c r="M8">
+        <v>0.05</v>
+      </c>
+      <c r="N8" t="s">
         <v>121</v>
       </c>
-      <c r="M8">
+      <c r="O8">
         <v>66</v>
       </c>
-      <c r="N8">
+      <c r="P8">
         <v>71</v>
       </c>
-      <c r="O8">
+      <c r="Q8">
         <v>93</v>
       </c>
-      <c r="P8" t="s">
-        <v>125</v>
-      </c>
-      <c r="Q8" t="s">
-        <v>129</v>
-      </c>
       <c r="R8" t="s">
-        <v>136</v>
+        <v>127</v>
       </c>
       <c r="S8" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="T8" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="U8" t="s">
-        <v>151</v>
+        <v>131</v>
+      </c>
+      <c r="V8" t="s">
+        <v>146</v>
+      </c>
+      <c r="W8" t="s">
+        <v>153</v>
+      </c>
+      <c r="X8">
+        <v>65</v>
+      </c>
+      <c r="Y8">
+        <v>35</v>
+      </c>
+      <c r="Z8">
+        <v>70</v>
+      </c>
+      <c r="AA8">
+        <v>0.25</v>
       </c>
     </row>
     <row r="9" spans="1:27">
@@ -1412,49 +1544,67 @@
         <v>13906.37</v>
       </c>
       <c r="G9" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="H9" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="I9" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="J9" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="K9" t="s">
+        <v>115</v>
+      </c>
+      <c r="L9" t="s">
         <v>117</v>
       </c>
-      <c r="L9" t="s">
-        <v>120</v>
-      </c>
       <c r="M9">
+        <v>0.05</v>
+      </c>
+      <c r="N9" t="s">
+        <v>121</v>
+      </c>
+      <c r="O9">
         <v>31</v>
       </c>
-      <c r="N9">
+      <c r="P9">
         <v>39</v>
       </c>
-      <c r="O9">
+      <c r="Q9">
         <v>81</v>
       </c>
-      <c r="P9" t="s">
-        <v>126</v>
-      </c>
-      <c r="Q9" t="s">
-        <v>129</v>
-      </c>
       <c r="R9" t="s">
-        <v>137</v>
+        <v>128</v>
       </c>
       <c r="S9" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="T9" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="U9" t="s">
-        <v>152</v>
+        <v>131</v>
+      </c>
+      <c r="V9" t="s">
+        <v>146</v>
+      </c>
+      <c r="W9" t="s">
+        <v>154</v>
+      </c>
+      <c r="X9">
+        <v>65</v>
+      </c>
+      <c r="Y9">
+        <v>35</v>
+      </c>
+      <c r="Z9">
+        <v>70</v>
+      </c>
+      <c r="AA9">
+        <v>0.25</v>
       </c>
     </row>
     <row r="10" spans="1:27">
@@ -1477,49 +1627,67 @@
         <v>29484.96</v>
       </c>
       <c r="G10" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="H10" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="I10" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="J10" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="K10" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="L10" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="M10">
+        <v>-0.5</v>
+      </c>
+      <c r="N10" t="s">
+        <v>122</v>
+      </c>
+      <c r="O10">
         <v>97</v>
       </c>
-      <c r="N10">
+      <c r="P10">
         <v>115</v>
       </c>
-      <c r="O10">
+      <c r="Q10">
         <v>85</v>
       </c>
-      <c r="P10" t="s">
-        <v>122</v>
-      </c>
-      <c r="Q10" t="s">
-        <v>129</v>
-      </c>
       <c r="R10" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="S10" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="T10" t="s">
-        <v>144</v>
+        <v>128</v>
       </c>
       <c r="U10" t="s">
-        <v>153</v>
+        <v>131</v>
+      </c>
+      <c r="V10" t="s">
+        <v>146</v>
+      </c>
+      <c r="W10" t="s">
+        <v>155</v>
+      </c>
+      <c r="X10">
+        <v>65</v>
+      </c>
+      <c r="Y10">
+        <v>35</v>
+      </c>
+      <c r="Z10">
+        <v>70</v>
+      </c>
+      <c r="AA10">
+        <v>0.25</v>
       </c>
     </row>
     <row r="11" spans="1:27">
@@ -1542,49 +1710,67 @@
         <v>30314.52</v>
       </c>
       <c r="G11" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="H11" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="I11" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="J11" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="K11" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="L11" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="M11">
+        <v>0.875</v>
+      </c>
+      <c r="N11" t="s">
+        <v>119</v>
+      </c>
+      <c r="O11">
         <v>172</v>
       </c>
-      <c r="N11">
+      <c r="P11">
         <v>200</v>
       </c>
-      <c r="O11">
+      <c r="Q11">
         <v>86</v>
       </c>
-      <c r="P11" t="s">
-        <v>126</v>
-      </c>
-      <c r="Q11" t="s">
-        <v>129</v>
-      </c>
       <c r="R11" t="s">
-        <v>138</v>
+        <v>128</v>
       </c>
       <c r="S11" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="T11" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="U11" t="s">
-        <v>154</v>
+        <v>131</v>
+      </c>
+      <c r="V11" t="s">
+        <v>146</v>
+      </c>
+      <c r="W11" t="s">
+        <v>156</v>
+      </c>
+      <c r="X11">
+        <v>65</v>
+      </c>
+      <c r="Y11">
+        <v>35</v>
+      </c>
+      <c r="Z11">
+        <v>70</v>
+      </c>
+      <c r="AA11">
+        <v>0.25</v>
       </c>
     </row>
     <row r="12" spans="1:27">
@@ -1607,49 +1793,67 @@
         <v>31368.74</v>
       </c>
       <c r="G12" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="H12" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="I12" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="J12" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="K12" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="L12" t="s">
+        <v>118</v>
+      </c>
+      <c r="M12">
+        <v>0.05</v>
+      </c>
+      <c r="N12" t="s">
         <v>121</v>
       </c>
-      <c r="M12">
+      <c r="O12">
         <v>33</v>
       </c>
-      <c r="N12">
+      <c r="P12">
         <v>37</v>
       </c>
-      <c r="O12">
+      <c r="Q12">
         <v>90</v>
       </c>
-      <c r="P12" t="s">
-        <v>127</v>
-      </c>
-      <c r="Q12" t="s">
+      <c r="R12" t="s">
         <v>129</v>
       </c>
-      <c r="R12" t="s">
-        <v>139</v>
-      </c>
       <c r="S12" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="T12" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="U12" t="s">
-        <v>155</v>
+        <v>131</v>
+      </c>
+      <c r="V12" t="s">
+        <v>146</v>
+      </c>
+      <c r="W12" t="s">
+        <v>157</v>
+      </c>
+      <c r="X12">
+        <v>65</v>
+      </c>
+      <c r="Y12">
+        <v>35</v>
+      </c>
+      <c r="Z12">
+        <v>70</v>
+      </c>
+      <c r="AA12">
+        <v>0.25</v>
       </c>
     </row>
     <row r="13" spans="1:27">
@@ -1672,49 +1876,67 @@
         <v>30990.38</v>
       </c>
       <c r="G13" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="H13" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="I13" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="J13" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="K13" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="L13" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="M13">
+        <v>0.55</v>
+      </c>
+      <c r="N13" t="s">
+        <v>120</v>
+      </c>
+      <c r="O13">
         <v>59</v>
       </c>
-      <c r="N13">
+      <c r="P13">
         <v>68</v>
       </c>
-      <c r="O13">
+      <c r="Q13">
         <v>87</v>
       </c>
-      <c r="P13" t="s">
-        <v>125</v>
-      </c>
-      <c r="Q13" t="s">
-        <v>129</v>
-      </c>
       <c r="R13" t="s">
-        <v>140</v>
+        <v>127</v>
       </c>
       <c r="S13" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="T13" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="U13" t="s">
-        <v>156</v>
+        <v>131</v>
+      </c>
+      <c r="V13" t="s">
+        <v>146</v>
+      </c>
+      <c r="W13" t="s">
+        <v>158</v>
+      </c>
+      <c r="X13">
+        <v>65</v>
+      </c>
+      <c r="Y13">
+        <v>35</v>
+      </c>
+      <c r="Z13">
+        <v>70</v>
+      </c>
+      <c r="AA13">
+        <v>0.25</v>
       </c>
     </row>
     <row r="14" spans="1:27">
@@ -1737,49 +1959,67 @@
         <v>11389.29</v>
       </c>
       <c r="G14" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="H14" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="I14" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="J14" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="K14" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="L14" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="M14">
+        <v>-0.875</v>
+      </c>
+      <c r="N14" t="s">
+        <v>123</v>
+      </c>
+      <c r="O14">
         <v>54</v>
       </c>
-      <c r="N14">
+      <c r="P14">
         <v>165</v>
       </c>
-      <c r="O14">
+      <c r="Q14">
         <v>33</v>
       </c>
-      <c r="P14" t="s">
-        <v>123</v>
-      </c>
-      <c r="Q14" t="s">
-        <v>129</v>
-      </c>
       <c r="R14" t="s">
-        <v>141</v>
+        <v>125</v>
       </c>
       <c r="S14" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="T14" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="U14" t="s">
-        <v>157</v>
+        <v>131</v>
+      </c>
+      <c r="V14" t="s">
+        <v>146</v>
+      </c>
+      <c r="W14" t="s">
+        <v>159</v>
+      </c>
+      <c r="X14">
+        <v>65</v>
+      </c>
+      <c r="Y14">
+        <v>35</v>
+      </c>
+      <c r="Z14">
+        <v>70</v>
+      </c>
+      <c r="AA14">
+        <v>0.25</v>
       </c>
     </row>
     <row r="15" spans="1:27">
@@ -1802,49 +2042,67 @@
         <v>10663.55</v>
       </c>
       <c r="G15" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="H15" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="I15" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="J15" t="s">
+        <v>112</v>
+      </c>
+      <c r="K15" t="s">
         <v>115</v>
       </c>
-      <c r="K15" t="s">
-        <v>117</v>
-      </c>
       <c r="L15" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="M15">
+        <v>-0.5</v>
+      </c>
+      <c r="N15" t="s">
+        <v>122</v>
+      </c>
+      <c r="O15">
         <v>30</v>
       </c>
-      <c r="N15">
+      <c r="P15">
         <v>46</v>
       </c>
-      <c r="O15">
+      <c r="Q15">
         <v>66</v>
       </c>
-      <c r="P15" t="s">
-        <v>126</v>
-      </c>
-      <c r="Q15" t="s">
-        <v>129</v>
-      </c>
       <c r="R15" t="s">
-        <v>142</v>
+        <v>128</v>
       </c>
       <c r="S15" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="T15" t="s">
         <v>144</v>
       </c>
       <c r="U15" t="s">
-        <v>158</v>
+        <v>131</v>
+      </c>
+      <c r="V15" t="s">
+        <v>146</v>
+      </c>
+      <c r="W15" t="s">
+        <v>160</v>
+      </c>
+      <c r="X15">
+        <v>65</v>
+      </c>
+      <c r="Y15">
+        <v>35</v>
+      </c>
+      <c r="Z15">
+        <v>70</v>
+      </c>
+      <c r="AA15">
+        <v>0.25</v>
       </c>
     </row>
     <row r="16" spans="1:27">
@@ -1867,49 +2125,67 @@
         <v>37182.71</v>
       </c>
       <c r="G16" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="H16" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="I16" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="J16" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="K16" t="s">
+        <v>115</v>
+      </c>
+      <c r="L16" t="s">
         <v>117</v>
       </c>
-      <c r="L16" t="s">
-        <v>120</v>
-      </c>
       <c r="M16">
+        <v>0.05</v>
+      </c>
+      <c r="N16" t="s">
+        <v>121</v>
+      </c>
+      <c r="O16">
         <v>70</v>
       </c>
-      <c r="N16">
+      <c r="P16">
         <v>191</v>
       </c>
-      <c r="O16">
+      <c r="Q16">
         <v>37</v>
       </c>
-      <c r="P16" t="s">
-        <v>128</v>
-      </c>
-      <c r="Q16" t="s">
-        <v>129</v>
-      </c>
       <c r="R16" t="s">
-        <v>143</v>
+        <v>130</v>
       </c>
       <c r="S16" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="T16" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="U16" t="s">
-        <v>159</v>
+        <v>131</v>
+      </c>
+      <c r="V16" t="s">
+        <v>146</v>
+      </c>
+      <c r="W16" t="s">
+        <v>161</v>
+      </c>
+      <c r="X16">
+        <v>65</v>
+      </c>
+      <c r="Y16">
+        <v>35</v>
+      </c>
+      <c r="Z16">
+        <v>70</v>
+      </c>
+      <c r="AA16">
+        <v>0.25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Enhance email functionality by adding endpoints for generating email previews and sending emails to individual accounts. Update the email scheduler to support personalized content generation. Include new dependencies in pyproject.toml and uv.lock for openpyxl and et-xmlfile. Refactor voice call handling to allow manual call triggers for specific accounts, improving user control over communication processes.
</commit_message>
<xml_diff>
--- a/data/test_dataset_15_accounts.xlsx
+++ b/data/test_dataset_15_accounts.xlsx
@@ -7,14 +7,14 @@
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="Accounts" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="282" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="135">
   <si>
     <t>name</t>
   </si>
@@ -241,87 +241,6 @@
     <t>Large</t>
   </si>
   <si>
-    <t>2025-02-21</t>
-  </si>
-  <si>
-    <t>2025-12-23</t>
-  </si>
-  <si>
-    <t>2026-01-02</t>
-  </si>
-  <si>
-    <t>2026-01-07</t>
-  </si>
-  <si>
-    <t>2025-08-25</t>
-  </si>
-  <si>
-    <t>2025-09-04</t>
-  </si>
-  <si>
-    <t>2025-09-14</t>
-  </si>
-  <si>
-    <t>2025-04-27</t>
-  </si>
-  <si>
-    <t>2025-05-07</t>
-  </si>
-  <si>
-    <t>2025-05-17</t>
-  </si>
-  <si>
-    <t>2025-05-27</t>
-  </si>
-  <si>
-    <t>2025-06-06</t>
-  </si>
-  <si>
-    <t>2025-06-16</t>
-  </si>
-  <si>
-    <t>2025-11-23</t>
-  </si>
-  <si>
-    <t>2026-01-22</t>
-  </si>
-  <si>
-    <t>2026-12-23</t>
-  </si>
-  <si>
-    <t>2027-01-02</t>
-  </si>
-  <si>
-    <t>2027-01-07</t>
-  </si>
-  <si>
-    <t>2026-08-25</t>
-  </si>
-  <si>
-    <t>2026-09-04</t>
-  </si>
-  <si>
-    <t>2026-09-14</t>
-  </si>
-  <si>
-    <t>2026-04-27</t>
-  </si>
-  <si>
-    <t>2026-05-07</t>
-  </si>
-  <si>
-    <t>2026-05-17</t>
-  </si>
-  <si>
-    <t>2026-05-27</t>
-  </si>
-  <si>
-    <t>2026-06-06</t>
-  </si>
-  <si>
-    <t>2026-06-16</t>
-  </si>
-  <si>
     <t>2026-01-28 15:24:16</t>
   </si>
   <si>
@@ -358,19 +277,19 @@
     <t>2026-02-14 15:24:16</t>
   </si>
   <si>
+    <t>active</t>
+  </si>
+  <si>
     <t>renewed</t>
   </si>
   <si>
-    <t>active</t>
+    <t>t90</t>
   </si>
   <si>
     <t>t60</t>
   </si>
   <si>
     <t>t30</t>
-  </si>
-  <si>
-    <t>t90</t>
   </si>
   <si>
     <t>very_positive</t>
@@ -506,6 +425,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <sz val="11"/>
@@ -558,11 +480,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -962,29 +885,29 @@
       <c r="F2">
         <v>29128.06</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" s="2">
+        <v>45769</v>
+      </c>
+      <c r="H2" s="2">
+        <v>46143</v>
+      </c>
+      <c r="I2" s="2">
+        <v>46143</v>
+      </c>
+      <c r="J2" t="s">
         <v>75</v>
       </c>
-      <c r="H2" t="s">
-        <v>88</v>
-      </c>
-      <c r="I2" t="s">
-        <v>88</v>
-      </c>
-      <c r="J2" t="s">
-        <v>102</v>
-      </c>
       <c r="K2" t="s">
-        <v>114</v>
+        <v>87</v>
       </c>
       <c r="L2" t="s">
-        <v>114</v>
+        <v>89</v>
       </c>
       <c r="M2">
         <v>0.875</v>
       </c>
       <c r="N2" t="s">
-        <v>119</v>
+        <v>92</v>
       </c>
       <c r="O2">
         <v>124</v>
@@ -996,34 +919,22 @@
         <v>89</v>
       </c>
       <c r="R2" t="s">
-        <v>124</v>
+        <v>97</v>
       </c>
       <c r="S2" t="s">
-        <v>131</v>
+        <v>104</v>
       </c>
       <c r="T2" t="s">
-        <v>132</v>
+        <v>105</v>
       </c>
       <c r="U2" t="s">
-        <v>131</v>
+        <v>104</v>
       </c>
       <c r="V2" t="s">
-        <v>146</v>
+        <v>119</v>
       </c>
       <c r="W2" t="s">
-        <v>147</v>
-      </c>
-      <c r="X2">
-        <v>65</v>
-      </c>
-      <c r="Y2">
-        <v>35</v>
-      </c>
-      <c r="Z2">
-        <v>70</v>
-      </c>
-      <c r="AA2">
-        <v>0.25</v>
+        <v>120</v>
       </c>
     </row>
     <row r="3" spans="1:27">
@@ -1045,29 +956,29 @@
       <c r="F3">
         <v>16600.38</v>
       </c>
-      <c r="G3" t="s">
-        <v>75</v>
-      </c>
-      <c r="H3" t="s">
+      <c r="G3" s="2">
+        <v>45769</v>
+      </c>
+      <c r="H3" s="2">
+        <v>46143</v>
+      </c>
+      <c r="I3" s="2">
+        <v>46143</v>
+      </c>
+      <c r="J3" t="s">
         <v>76</v>
       </c>
-      <c r="I3" t="s">
-        <v>76</v>
-      </c>
-      <c r="J3" t="s">
-        <v>103</v>
-      </c>
       <c r="K3" t="s">
-        <v>114</v>
+        <v>87</v>
       </c>
       <c r="L3" t="s">
-        <v>116</v>
+        <v>89</v>
       </c>
       <c r="M3">
         <v>0.55</v>
       </c>
       <c r="N3" t="s">
-        <v>120</v>
+        <v>93</v>
       </c>
       <c r="O3">
         <v>143</v>
@@ -1079,34 +990,22 @@
         <v>85</v>
       </c>
       <c r="R3" t="s">
-        <v>125</v>
+        <v>98</v>
       </c>
       <c r="S3" t="s">
-        <v>131</v>
+        <v>104</v>
       </c>
       <c r="T3" t="s">
-        <v>133</v>
+        <v>106</v>
       </c>
       <c r="U3" t="s">
-        <v>131</v>
+        <v>104</v>
       </c>
       <c r="V3" t="s">
-        <v>146</v>
+        <v>119</v>
       </c>
       <c r="W3" t="s">
-        <v>148</v>
-      </c>
-      <c r="X3">
-        <v>65</v>
-      </c>
-      <c r="Y3">
-        <v>35</v>
-      </c>
-      <c r="Z3">
-        <v>70</v>
-      </c>
-      <c r="AA3">
-        <v>0.25</v>
+        <v>121</v>
       </c>
     </row>
     <row r="4" spans="1:27">
@@ -1128,29 +1027,29 @@
       <c r="F4">
         <v>16100.95</v>
       </c>
-      <c r="G4" t="s">
-        <v>75</v>
-      </c>
-      <c r="H4" t="s">
+      <c r="G4" s="2">
+        <v>45769</v>
+      </c>
+      <c r="H4" s="2">
+        <v>46143</v>
+      </c>
+      <c r="I4" s="2">
+        <v>46143</v>
+      </c>
+      <c r="J4" t="s">
+        <v>77</v>
+      </c>
+      <c r="K4" t="s">
+        <v>87</v>
+      </c>
+      <c r="L4" t="s">
         <v>89</v>
-      </c>
-      <c r="I4" t="s">
-        <v>89</v>
-      </c>
-      <c r="J4" t="s">
-        <v>104</v>
-      </c>
-      <c r="K4" t="s">
-        <v>114</v>
-      </c>
-      <c r="L4" t="s">
-        <v>117</v>
       </c>
       <c r="M4">
         <v>0.05</v>
       </c>
       <c r="N4" t="s">
-        <v>121</v>
+        <v>94</v>
       </c>
       <c r="O4">
         <v>140</v>
@@ -1162,34 +1061,22 @@
         <v>86</v>
       </c>
       <c r="R4" t="s">
-        <v>126</v>
+        <v>99</v>
       </c>
       <c r="S4" t="s">
-        <v>131</v>
+        <v>104</v>
       </c>
       <c r="T4" t="s">
-        <v>134</v>
+        <v>107</v>
       </c>
       <c r="U4" t="s">
-        <v>131</v>
+        <v>104</v>
       </c>
       <c r="V4" t="s">
-        <v>146</v>
+        <v>119</v>
       </c>
       <c r="W4" t="s">
-        <v>149</v>
-      </c>
-      <c r="X4">
-        <v>65</v>
-      </c>
-      <c r="Y4">
-        <v>35</v>
-      </c>
-      <c r="Z4">
-        <v>70</v>
-      </c>
-      <c r="AA4">
-        <v>0.25</v>
+        <v>122</v>
       </c>
     </row>
     <row r="5" spans="1:27">
@@ -1211,29 +1098,29 @@
       <c r="F5">
         <v>29607.6</v>
       </c>
-      <c r="G5" t="s">
-        <v>76</v>
-      </c>
-      <c r="H5" t="s">
-        <v>90</v>
-      </c>
-      <c r="I5" t="s">
-        <v>90</v>
+      <c r="G5" s="2">
+        <v>45769</v>
+      </c>
+      <c r="H5" s="2">
+        <v>46143</v>
+      </c>
+      <c r="I5" s="2">
+        <v>46143</v>
       </c>
       <c r="J5" t="s">
-        <v>105</v>
+        <v>78</v>
       </c>
       <c r="K5" t="s">
-        <v>115</v>
+        <v>87</v>
       </c>
       <c r="L5" t="s">
-        <v>117</v>
+        <v>89</v>
       </c>
       <c r="M5">
         <v>-0.5</v>
       </c>
       <c r="N5" t="s">
-        <v>122</v>
+        <v>95</v>
       </c>
       <c r="O5">
         <v>36</v>
@@ -1245,34 +1132,22 @@
         <v>72</v>
       </c>
       <c r="R5" t="s">
-        <v>126</v>
+        <v>99</v>
       </c>
       <c r="S5" t="s">
-        <v>131</v>
+        <v>104</v>
       </c>
       <c r="T5" t="s">
-        <v>135</v>
+        <v>108</v>
       </c>
       <c r="U5" t="s">
-        <v>131</v>
+        <v>104</v>
       </c>
       <c r="V5" t="s">
-        <v>146</v>
+        <v>119</v>
       </c>
       <c r="W5" t="s">
-        <v>150</v>
-      </c>
-      <c r="X5">
-        <v>65</v>
-      </c>
-      <c r="Y5">
-        <v>35</v>
-      </c>
-      <c r="Z5">
-        <v>70</v>
-      </c>
-      <c r="AA5">
-        <v>0.25</v>
+        <v>123</v>
       </c>
     </row>
     <row r="6" spans="1:27">
@@ -1294,29 +1169,29 @@
       <c r="F6">
         <v>41528.6</v>
       </c>
-      <c r="G6" t="s">
-        <v>77</v>
-      </c>
-      <c r="H6" t="s">
-        <v>91</v>
-      </c>
-      <c r="I6" t="s">
-        <v>91</v>
+      <c r="G6" s="2">
+        <v>45901</v>
+      </c>
+      <c r="H6" s="2">
+        <v>46266</v>
+      </c>
+      <c r="I6" s="2">
+        <v>46266</v>
       </c>
       <c r="J6" t="s">
-        <v>106</v>
+        <v>79</v>
       </c>
       <c r="K6" t="s">
-        <v>115</v>
+        <v>87</v>
       </c>
       <c r="L6" t="s">
-        <v>114</v>
+        <v>90</v>
       </c>
       <c r="M6">
         <v>-0.875</v>
       </c>
       <c r="N6" t="s">
-        <v>123</v>
+        <v>96</v>
       </c>
       <c r="O6">
         <v>70</v>
@@ -1328,34 +1203,22 @@
         <v>62</v>
       </c>
       <c r="R6" t="s">
-        <v>125</v>
+        <v>98</v>
       </c>
       <c r="S6" t="s">
-        <v>131</v>
+        <v>104</v>
       </c>
       <c r="T6" t="s">
-        <v>136</v>
+        <v>109</v>
       </c>
       <c r="U6" t="s">
-        <v>131</v>
+        <v>104</v>
       </c>
       <c r="V6" t="s">
-        <v>146</v>
+        <v>119</v>
       </c>
       <c r="W6" t="s">
-        <v>151</v>
-      </c>
-      <c r="X6">
-        <v>65</v>
-      </c>
-      <c r="Y6">
-        <v>35</v>
-      </c>
-      <c r="Z6">
-        <v>70</v>
-      </c>
-      <c r="AA6">
-        <v>0.25</v>
+        <v>124</v>
       </c>
     </row>
     <row r="7" spans="1:27">
@@ -1377,29 +1240,29 @@
       <c r="F7">
         <v>1622.41</v>
       </c>
-      <c r="G7" t="s">
+      <c r="G7" s="2">
+        <v>45901</v>
+      </c>
+      <c r="H7" s="2">
+        <v>46266</v>
+      </c>
+      <c r="I7" s="2">
+        <v>46266</v>
+      </c>
+      <c r="J7" t="s">
         <v>78</v>
       </c>
-      <c r="H7" t="s">
-        <v>92</v>
-      </c>
-      <c r="I7" t="s">
-        <v>92</v>
-      </c>
-      <c r="J7" t="s">
-        <v>105</v>
-      </c>
       <c r="K7" t="s">
-        <v>115</v>
+        <v>87</v>
       </c>
       <c r="L7" t="s">
-        <v>117</v>
+        <v>90</v>
       </c>
       <c r="M7">
         <v>0.55</v>
       </c>
       <c r="N7" t="s">
-        <v>120</v>
+        <v>93</v>
       </c>
       <c r="O7">
         <v>47</v>
@@ -1411,34 +1274,22 @@
         <v>44</v>
       </c>
       <c r="R7" t="s">
-        <v>124</v>
+        <v>97</v>
       </c>
       <c r="S7" t="s">
-        <v>131</v>
+        <v>104</v>
       </c>
       <c r="T7" t="s">
-        <v>137</v>
+        <v>110</v>
       </c>
       <c r="U7" t="s">
-        <v>131</v>
+        <v>104</v>
       </c>
       <c r="V7" t="s">
-        <v>146</v>
+        <v>119</v>
       </c>
       <c r="W7" t="s">
-        <v>152</v>
-      </c>
-      <c r="X7">
-        <v>65</v>
-      </c>
-      <c r="Y7">
-        <v>35</v>
-      </c>
-      <c r="Z7">
-        <v>70</v>
-      </c>
-      <c r="AA7">
-        <v>0.25</v>
+        <v>125</v>
       </c>
     </row>
     <row r="8" spans="1:27">
@@ -1460,29 +1311,29 @@
       <c r="F8">
         <v>20954.26</v>
       </c>
-      <c r="G8" t="s">
-        <v>79</v>
-      </c>
-      <c r="H8" t="s">
-        <v>93</v>
-      </c>
-      <c r="I8" t="s">
-        <v>93</v>
+      <c r="G8" s="2">
+        <v>45901</v>
+      </c>
+      <c r="H8" s="2">
+        <v>46266</v>
+      </c>
+      <c r="I8" s="2">
+        <v>46266</v>
       </c>
       <c r="J8" t="s">
-        <v>107</v>
+        <v>80</v>
       </c>
       <c r="K8" t="s">
-        <v>115</v>
+        <v>87</v>
       </c>
       <c r="L8" t="s">
-        <v>118</v>
+        <v>90</v>
       </c>
       <c r="M8">
         <v>0.05</v>
       </c>
       <c r="N8" t="s">
-        <v>121</v>
+        <v>94</v>
       </c>
       <c r="O8">
         <v>66</v>
@@ -1494,34 +1345,22 @@
         <v>93</v>
       </c>
       <c r="R8" t="s">
-        <v>127</v>
+        <v>100</v>
       </c>
       <c r="S8" t="s">
-        <v>131</v>
+        <v>104</v>
       </c>
       <c r="T8" t="s">
-        <v>138</v>
+        <v>111</v>
       </c>
       <c r="U8" t="s">
-        <v>131</v>
+        <v>104</v>
       </c>
       <c r="V8" t="s">
-        <v>146</v>
+        <v>119</v>
       </c>
       <c r="W8" t="s">
-        <v>153</v>
-      </c>
-      <c r="X8">
-        <v>65</v>
-      </c>
-      <c r="Y8">
-        <v>35</v>
-      </c>
-      <c r="Z8">
-        <v>70</v>
-      </c>
-      <c r="AA8">
-        <v>0.25</v>
+        <v>126</v>
       </c>
     </row>
     <row r="9" spans="1:27">
@@ -1543,29 +1382,29 @@
       <c r="F9">
         <v>13906.37</v>
       </c>
-      <c r="G9" t="s">
-        <v>80</v>
-      </c>
-      <c r="H9" t="s">
-        <v>94</v>
-      </c>
-      <c r="I9" t="s">
-        <v>94</v>
+      <c r="G9" s="2">
+        <v>45901</v>
+      </c>
+      <c r="H9" s="2">
+        <v>46266</v>
+      </c>
+      <c r="I9" s="2">
+        <v>46266</v>
       </c>
       <c r="J9" t="s">
-        <v>108</v>
+        <v>81</v>
       </c>
       <c r="K9" t="s">
-        <v>115</v>
+        <v>87</v>
       </c>
       <c r="L9" t="s">
-        <v>117</v>
+        <v>90</v>
       </c>
       <c r="M9">
         <v>0.05</v>
       </c>
       <c r="N9" t="s">
-        <v>121</v>
+        <v>94</v>
       </c>
       <c r="O9">
         <v>31</v>
@@ -1577,34 +1416,22 @@
         <v>81</v>
       </c>
       <c r="R9" t="s">
-        <v>128</v>
+        <v>101</v>
       </c>
       <c r="S9" t="s">
-        <v>131</v>
+        <v>104</v>
       </c>
       <c r="T9" t="s">
-        <v>139</v>
+        <v>112</v>
       </c>
       <c r="U9" t="s">
-        <v>131</v>
+        <v>104</v>
       </c>
       <c r="V9" t="s">
-        <v>146</v>
+        <v>119</v>
       </c>
       <c r="W9" t="s">
-        <v>154</v>
-      </c>
-      <c r="X9">
-        <v>65</v>
-      </c>
-      <c r="Y9">
-        <v>35</v>
-      </c>
-      <c r="Z9">
-        <v>70</v>
-      </c>
-      <c r="AA9">
-        <v>0.25</v>
+        <v>127</v>
       </c>
     </row>
     <row r="10" spans="1:27">
@@ -1626,29 +1453,29 @@
       <c r="F10">
         <v>29484.96</v>
       </c>
-      <c r="G10" t="s">
-        <v>81</v>
-      </c>
-      <c r="H10" t="s">
-        <v>95</v>
-      </c>
-      <c r="I10" t="s">
-        <v>95</v>
+      <c r="G10" s="2">
+        <v>45998</v>
+      </c>
+      <c r="H10" s="2">
+        <v>46363</v>
+      </c>
+      <c r="I10" s="2">
+        <v>46363</v>
       </c>
       <c r="J10" t="s">
-        <v>109</v>
+        <v>82</v>
       </c>
       <c r="K10" t="s">
-        <v>115</v>
+        <v>87</v>
       </c>
       <c r="L10" t="s">
-        <v>114</v>
+        <v>91</v>
       </c>
       <c r="M10">
         <v>-0.5</v>
       </c>
       <c r="N10" t="s">
-        <v>122</v>
+        <v>95</v>
       </c>
       <c r="O10">
         <v>97</v>
@@ -1660,34 +1487,22 @@
         <v>85</v>
       </c>
       <c r="R10" t="s">
-        <v>124</v>
+        <v>97</v>
       </c>
       <c r="S10" t="s">
-        <v>131</v>
+        <v>104</v>
       </c>
       <c r="T10" t="s">
+        <v>101</v>
+      </c>
+      <c r="U10" t="s">
+        <v>104</v>
+      </c>
+      <c r="V10" t="s">
+        <v>119</v>
+      </c>
+      <c r="W10" t="s">
         <v>128</v>
-      </c>
-      <c r="U10" t="s">
-        <v>131</v>
-      </c>
-      <c r="V10" t="s">
-        <v>146</v>
-      </c>
-      <c r="W10" t="s">
-        <v>155</v>
-      </c>
-      <c r="X10">
-        <v>65</v>
-      </c>
-      <c r="Y10">
-        <v>35</v>
-      </c>
-      <c r="Z10">
-        <v>70</v>
-      </c>
-      <c r="AA10">
-        <v>0.25</v>
       </c>
     </row>
     <row r="11" spans="1:27">
@@ -1709,29 +1524,29 @@
       <c r="F11">
         <v>30314.52</v>
       </c>
-      <c r="G11" t="s">
-        <v>82</v>
-      </c>
-      <c r="H11" t="s">
-        <v>96</v>
-      </c>
-      <c r="I11" t="s">
-        <v>96</v>
+      <c r="G11" s="2">
+        <v>45998</v>
+      </c>
+      <c r="H11" s="2">
+        <v>46363</v>
+      </c>
+      <c r="I11" s="2">
+        <v>46363</v>
       </c>
       <c r="J11" t="s">
-        <v>104</v>
+        <v>77</v>
       </c>
       <c r="K11" t="s">
-        <v>115</v>
+        <v>87</v>
       </c>
       <c r="L11" t="s">
-        <v>118</v>
+        <v>91</v>
       </c>
       <c r="M11">
         <v>0.875</v>
       </c>
       <c r="N11" t="s">
-        <v>119</v>
+        <v>92</v>
       </c>
       <c r="O11">
         <v>172</v>
@@ -1743,34 +1558,22 @@
         <v>86</v>
       </c>
       <c r="R11" t="s">
-        <v>128</v>
+        <v>101</v>
       </c>
       <c r="S11" t="s">
-        <v>131</v>
+        <v>104</v>
       </c>
       <c r="T11" t="s">
-        <v>140</v>
+        <v>113</v>
       </c>
       <c r="U11" t="s">
-        <v>131</v>
+        <v>104</v>
       </c>
       <c r="V11" t="s">
-        <v>146</v>
+        <v>119</v>
       </c>
       <c r="W11" t="s">
-        <v>156</v>
-      </c>
-      <c r="X11">
-        <v>65</v>
-      </c>
-      <c r="Y11">
-        <v>35</v>
-      </c>
-      <c r="Z11">
-        <v>70</v>
-      </c>
-      <c r="AA11">
-        <v>0.25</v>
+        <v>129</v>
       </c>
     </row>
     <row r="12" spans="1:27">
@@ -1792,29 +1595,29 @@
       <c r="F12">
         <v>31368.74</v>
       </c>
-      <c r="G12" t="s">
+      <c r="G12" s="2">
+        <v>45998</v>
+      </c>
+      <c r="H12" s="2">
+        <v>46363</v>
+      </c>
+      <c r="I12" s="2">
+        <v>46363</v>
+      </c>
+      <c r="J12" t="s">
         <v>83</v>
       </c>
-      <c r="H12" t="s">
-        <v>97</v>
-      </c>
-      <c r="I12" t="s">
-        <v>97</v>
-      </c>
-      <c r="J12" t="s">
-        <v>110</v>
-      </c>
       <c r="K12" t="s">
-        <v>115</v>
+        <v>87</v>
       </c>
       <c r="L12" t="s">
-        <v>118</v>
+        <v>91</v>
       </c>
       <c r="M12">
         <v>0.05</v>
       </c>
       <c r="N12" t="s">
-        <v>121</v>
+        <v>94</v>
       </c>
       <c r="O12">
         <v>33</v>
@@ -1826,34 +1629,22 @@
         <v>90</v>
       </c>
       <c r="R12" t="s">
-        <v>129</v>
+        <v>102</v>
       </c>
       <c r="S12" t="s">
-        <v>131</v>
+        <v>104</v>
       </c>
       <c r="T12" t="s">
-        <v>141</v>
+        <v>114</v>
       </c>
       <c r="U12" t="s">
-        <v>131</v>
+        <v>104</v>
       </c>
       <c r="V12" t="s">
-        <v>146</v>
+        <v>119</v>
       </c>
       <c r="W12" t="s">
-        <v>157</v>
-      </c>
-      <c r="X12">
-        <v>65</v>
-      </c>
-      <c r="Y12">
-        <v>35</v>
-      </c>
-      <c r="Z12">
-        <v>70</v>
-      </c>
-      <c r="AA12">
-        <v>0.25</v>
+        <v>130</v>
       </c>
     </row>
     <row r="13" spans="1:27">
@@ -1875,29 +1666,29 @@
       <c r="F13">
         <v>30990.38</v>
       </c>
-      <c r="G13" t="s">
+      <c r="G13" s="2">
+        <v>45998</v>
+      </c>
+      <c r="H13" s="2">
+        <v>46363</v>
+      </c>
+      <c r="I13" s="2">
+        <v>46363</v>
+      </c>
+      <c r="J13" t="s">
         <v>84</v>
       </c>
-      <c r="H13" t="s">
-        <v>98</v>
-      </c>
-      <c r="I13" t="s">
-        <v>98</v>
-      </c>
-      <c r="J13" t="s">
-        <v>111</v>
-      </c>
       <c r="K13" t="s">
-        <v>115</v>
+        <v>87</v>
       </c>
       <c r="L13" t="s">
-        <v>116</v>
+        <v>91</v>
       </c>
       <c r="M13">
         <v>0.55</v>
       </c>
       <c r="N13" t="s">
-        <v>120</v>
+        <v>93</v>
       </c>
       <c r="O13">
         <v>59</v>
@@ -1909,34 +1700,22 @@
         <v>87</v>
       </c>
       <c r="R13" t="s">
-        <v>127</v>
+        <v>100</v>
       </c>
       <c r="S13" t="s">
+        <v>104</v>
+      </c>
+      <c r="T13" t="s">
+        <v>115</v>
+      </c>
+      <c r="U13" t="s">
+        <v>104</v>
+      </c>
+      <c r="V13" t="s">
+        <v>119</v>
+      </c>
+      <c r="W13" t="s">
         <v>131</v>
-      </c>
-      <c r="T13" t="s">
-        <v>142</v>
-      </c>
-      <c r="U13" t="s">
-        <v>131</v>
-      </c>
-      <c r="V13" t="s">
-        <v>146</v>
-      </c>
-      <c r="W13" t="s">
-        <v>158</v>
-      </c>
-      <c r="X13">
-        <v>65</v>
-      </c>
-      <c r="Y13">
-        <v>35</v>
-      </c>
-      <c r="Z13">
-        <v>70</v>
-      </c>
-      <c r="AA13">
-        <v>0.25</v>
       </c>
     </row>
     <row r="14" spans="1:27">
@@ -1958,29 +1737,29 @@
       <c r="F14">
         <v>11389.29</v>
       </c>
-      <c r="G14" t="s">
-        <v>85</v>
-      </c>
-      <c r="H14" t="s">
-        <v>99</v>
-      </c>
-      <c r="I14" t="s">
-        <v>99</v>
+      <c r="G14" s="2">
+        <v>45709</v>
+      </c>
+      <c r="H14" s="2">
+        <v>46037</v>
+      </c>
+      <c r="I14" s="2">
+        <v>46037</v>
       </c>
       <c r="J14" t="s">
-        <v>104</v>
+        <v>77</v>
       </c>
       <c r="K14" t="s">
-        <v>115</v>
+        <v>88</v>
       </c>
       <c r="L14" t="s">
-        <v>118</v>
+        <v>88</v>
       </c>
       <c r="M14">
         <v>-0.875</v>
       </c>
       <c r="N14" t="s">
-        <v>123</v>
+        <v>96</v>
       </c>
       <c r="O14">
         <v>54</v>
@@ -1992,34 +1771,22 @@
         <v>33</v>
       </c>
       <c r="R14" t="s">
-        <v>125</v>
+        <v>98</v>
       </c>
       <c r="S14" t="s">
-        <v>131</v>
+        <v>104</v>
       </c>
       <c r="T14" t="s">
-        <v>143</v>
+        <v>116</v>
       </c>
       <c r="U14" t="s">
-        <v>131</v>
+        <v>104</v>
       </c>
       <c r="V14" t="s">
-        <v>146</v>
+        <v>119</v>
       </c>
       <c r="W14" t="s">
-        <v>159</v>
-      </c>
-      <c r="X14">
-        <v>65</v>
-      </c>
-      <c r="Y14">
-        <v>35</v>
-      </c>
-      <c r="Z14">
-        <v>70</v>
-      </c>
-      <c r="AA14">
-        <v>0.25</v>
+        <v>132</v>
       </c>
     </row>
     <row r="15" spans="1:27">
@@ -2041,29 +1808,29 @@
       <c r="F15">
         <v>10663.55</v>
       </c>
-      <c r="G15" t="s">
-        <v>86</v>
-      </c>
-      <c r="H15" t="s">
-        <v>100</v>
-      </c>
-      <c r="I15" t="s">
-        <v>100</v>
+      <c r="G15" s="2">
+        <v>45709</v>
+      </c>
+      <c r="H15" s="2">
+        <v>46037</v>
+      </c>
+      <c r="I15" s="2">
+        <v>46037</v>
       </c>
       <c r="J15" t="s">
-        <v>112</v>
+        <v>85</v>
       </c>
       <c r="K15" t="s">
-        <v>115</v>
+        <v>88</v>
       </c>
       <c r="L15" t="s">
-        <v>116</v>
+        <v>88</v>
       </c>
       <c r="M15">
         <v>-0.5</v>
       </c>
       <c r="N15" t="s">
-        <v>122</v>
+        <v>95</v>
       </c>
       <c r="O15">
         <v>30</v>
@@ -2075,34 +1842,22 @@
         <v>66</v>
       </c>
       <c r="R15" t="s">
-        <v>128</v>
+        <v>101</v>
       </c>
       <c r="S15" t="s">
-        <v>131</v>
+        <v>104</v>
       </c>
       <c r="T15" t="s">
-        <v>144</v>
+        <v>117</v>
       </c>
       <c r="U15" t="s">
-        <v>131</v>
+        <v>104</v>
       </c>
       <c r="V15" t="s">
-        <v>146</v>
+        <v>119</v>
       </c>
       <c r="W15" t="s">
-        <v>160</v>
-      </c>
-      <c r="X15">
-        <v>65</v>
-      </c>
-      <c r="Y15">
-        <v>35</v>
-      </c>
-      <c r="Z15">
-        <v>70</v>
-      </c>
-      <c r="AA15">
-        <v>0.25</v>
+        <v>133</v>
       </c>
     </row>
     <row r="16" spans="1:27">
@@ -2124,29 +1879,29 @@
       <c r="F16">
         <v>37182.71</v>
       </c>
-      <c r="G16" t="s">
-        <v>87</v>
-      </c>
-      <c r="H16" t="s">
-        <v>101</v>
-      </c>
-      <c r="I16" t="s">
-        <v>101</v>
+      <c r="G16" s="2">
+        <v>45709</v>
+      </c>
+      <c r="H16" s="2">
+        <v>46037</v>
+      </c>
+      <c r="I16" s="2">
+        <v>46037</v>
       </c>
       <c r="J16" t="s">
-        <v>113</v>
+        <v>86</v>
       </c>
       <c r="K16" t="s">
-        <v>115</v>
+        <v>88</v>
       </c>
       <c r="L16" t="s">
-        <v>117</v>
+        <v>88</v>
       </c>
       <c r="M16">
         <v>0.05</v>
       </c>
       <c r="N16" t="s">
-        <v>121</v>
+        <v>94</v>
       </c>
       <c r="O16">
         <v>70</v>
@@ -2158,34 +1913,22 @@
         <v>37</v>
       </c>
       <c r="R16" t="s">
-        <v>130</v>
+        <v>103</v>
       </c>
       <c r="S16" t="s">
-        <v>131</v>
+        <v>104</v>
       </c>
       <c r="T16" t="s">
-        <v>145</v>
+        <v>118</v>
       </c>
       <c r="U16" t="s">
-        <v>131</v>
+        <v>104</v>
       </c>
       <c r="V16" t="s">
-        <v>146</v>
+        <v>119</v>
       </c>
       <c r="W16" t="s">
-        <v>161</v>
-      </c>
-      <c r="X16">
-        <v>65</v>
-      </c>
-      <c r="Y16">
-        <v>35</v>
-      </c>
-      <c r="Z16">
-        <v>70</v>
-      </c>
-      <c r="AA16">
-        <v>0.25</v>
+        <v>134</v>
       </c>
     </row>
   </sheetData>

</xml_diff>